<commit_message>
Add credit-cards product template with hero, cards, and accordion blocks
The credit-cards page was mis-mapped to the calculator-form-carousel
template, whose selectors didn't match, so it rendered as one flat block
of default content. Give it a dedicated product-page template mapping the
hero carousel, product/testimonial/offer card grids, and FAQ/info
accordions to existing blocks. Extend the cards-feature parser for
product-card (.mf-sm-cards) and offer (.offer-container) markup, and the
accordion-rates parser for flat h2.target + .toggle-ctnt structure. Scope
the homepage 6-card cap to image-bearing grids so the 12-item offers strip
shows fully.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-kotak.report.xlsx
+++ b/tools/importer/reports/import-kotak.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="553">
   <si>
     <t>_reportFile</t>
   </si>
@@ -1489,10 +1489,16 @@
     <t>en/personal-banking/cards/credit-cards.report.json</t>
   </si>
   <si>
+    <t>["carousel-banner","cards-feature","cards-feature","cards-feature","accordion-rates","accordion-rates"]</t>
+  </si>
+  <si>
     <t>en/personal-banking/cards/credit-cards</t>
   </si>
   <si>
-    <t>2026-06-19T08:38:50.108Z</t>
+    <t>credit-cards-product</t>
+  </si>
+  <si>
+    <t>2026-06-21T08:39:33.777Z</t>
   </si>
   <si>
     <t>Credit Card - Apply for Credit Card Online &amp; Get Instant Approval</t>
@@ -4380,36 +4386,36 @@
         <v>491</v>
       </c>
       <c r="B90" t="s">
-        <v>17</v>
+        <v>492</v>
       </c>
       <c r="C90" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D90" t="s">
         <v>11</v>
       </c>
       <c r="E90" t="s">
-        <v>36</v>
+        <v>494</v>
       </c>
       <c r="F90" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="G90" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="H90" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B91" t="s">
         <v>17</v>
       </c>
       <c r="C91" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="D91" t="s">
         <v>11</v>
@@ -4418,24 +4424,24 @@
         <v>12</v>
       </c>
       <c r="F91" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="G91" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="H91" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B92" t="s">
         <v>380</v>
       </c>
       <c r="C92" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D92" t="s">
         <v>11</v>
@@ -4444,24 +4450,24 @@
         <v>382</v>
       </c>
       <c r="F92" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="G92" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="H92" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B93" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C93" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D93" t="s">
         <v>11</v>
@@ -4470,24 +4476,24 @@
         <v>247</v>
       </c>
       <c r="F93" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="G93" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="H93" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B94" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C94" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D94" t="s">
         <v>11</v>
@@ -4496,24 +4502,24 @@
         <v>247</v>
       </c>
       <c r="F94" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="G94" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="H94" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B95" t="s">
         <v>17</v>
       </c>
       <c r="C95" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D95" t="s">
         <v>11</v>
@@ -4522,24 +4528,24 @@
         <v>103</v>
       </c>
       <c r="F95" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G95" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="H95" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B96" t="s">
         <v>17</v>
       </c>
       <c r="C96" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D96" t="s">
         <v>11</v>
@@ -4548,50 +4554,50 @@
         <v>103</v>
       </c>
       <c r="F96" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="G96" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="H96" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B97" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="C97" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D97" t="s">
         <v>11</v>
       </c>
       <c r="E97" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F97" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="G97" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="H97" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B98" t="s">
         <v>17</v>
       </c>
       <c r="C98" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D98" t="s">
         <v>11</v>
@@ -4600,24 +4606,24 @@
         <v>12</v>
       </c>
       <c r="F98" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="G98" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="H98" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B99" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="C99" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D99" t="s">
         <v>11</v>
@@ -4626,24 +4632,24 @@
         <v>247</v>
       </c>
       <c r="F99" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="G99" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="H99" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B100" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C100" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D100" t="s">
         <v>11</v>
@@ -4652,13 +4658,13 @@
         <v>176</v>
       </c>
       <c r="F100" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="G100" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="H100" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>

</xml_diff>